<commit_message>
chore: weekly briefing 2026-09-25 23:00Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-09-21.xlsx
+++ b/public/reports/weekly_briefing/2026-09-21.xlsx
@@ -1028,7 +1028,7 @@
       <c r="G6" s="3" t="inlineStr"/>
       <c r="H6" s="18" t="inlineStr">
         <is>
-          <t>미국 종가 기준 09/18 → 09/23, %</t>
+          <t>미국 종가 기준 09/18 → 09/25, %</t>
         </is>
       </c>
       <c r="I6" s="18" t="inlineStr"/>
@@ -1098,19 +1098,19 @@
         <v>16901</v>
       </c>
       <c r="E8" s="29" t="n">
-        <v>0.73</v>
-      </c>
-      <c r="F8" s="28" t="n">
-        <v>-0.33</v>
+        <v>1.21</v>
+      </c>
+      <c r="F8" s="29" t="n">
+        <v>0.28</v>
       </c>
       <c r="G8" s="29" t="n">
-        <v>1.56</v>
+        <v>2.06</v>
       </c>
       <c r="H8" s="29" t="n">
-        <v>6.68</v>
+        <v>0.41</v>
       </c>
       <c r="I8" s="29" t="n">
-        <v>5.14</v>
+        <v>6.27</v>
       </c>
     </row>
     <row r="9">
@@ -1169,7 +1169,7 @@
         </is>
       </c>
       <c r="D12" s="32" t="n">
-        <v>4.96</v>
+        <v>5.86</v>
       </c>
     </row>
     <row r="13">
@@ -1189,7 +1189,7 @@
         </is>
       </c>
       <c r="D13" s="32" t="n">
-        <v>3.15</v>
+        <v>3.64</v>
       </c>
     </row>
     <row r="14">
@@ -1205,11 +1205,11 @@
       </c>
       <c r="C14" s="31" t="inlineStr">
         <is>
-          <t>소재</t>
+          <t>헬스케어</t>
         </is>
       </c>
       <c r="D14" s="32" t="n">
-        <v>1.04</v>
+        <v>1.76</v>
       </c>
     </row>
     <row r="15">
@@ -1229,7 +1229,7 @@
         </is>
       </c>
       <c r="D15" s="33" t="n">
-        <v>-2.44</v>
+        <v>-2.96</v>
       </c>
     </row>
     <row r="16">
@@ -1249,7 +1249,7 @@
         </is>
       </c>
       <c r="D16" s="33" t="n">
-        <v>-2.02</v>
+        <v>-1.48</v>
       </c>
     </row>
     <row r="17">
@@ -1269,7 +1269,7 @@
         </is>
       </c>
       <c r="D17" s="33" t="n">
-        <v>-0.97</v>
+        <v>-1.08</v>
       </c>
     </row>
     <row r="18">
@@ -11252,7 +11252,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{9DA787CD-8A5E-4F13-8D53-539D4FE166AF}</x14:id>
+          <x14:id>{3F13C55D-0746-4EC0-8B69-BBDC340D7B12}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11266,7 +11266,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{B4B60FBA-AA05-4E50-9168-9EC719FAD6E7}</x14:id>
+          <x14:id>{4896E0A4-6A93-4372-B48D-565D1EA8ACAB}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11280,7 +11280,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0D036BDC-A79A-4A0C-96A1-3BC607F585D6}</x14:id>
+          <x14:id>{75A179DD-CD7C-467D-BFEC-3EB09BAEC858}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11294,7 +11294,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D42676F0-B450-4A68-A5EA-A761A52DBE84}</x14:id>
+          <x14:id>{9797D8CE-C476-481A-88E1-78D483D0FE4B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11304,7 +11304,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{9DA787CD-8A5E-4F13-8D53-539D4FE166AF}">
+          <x14:cfRule type="dataBar" id="{3F13C55D-0746-4EC0-8B69-BBDC340D7B12}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11317,7 +11317,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{B4B60FBA-AA05-4E50-9168-9EC719FAD6E7}">
+          <x14:cfRule type="dataBar" id="{4896E0A4-6A93-4372-B48D-565D1EA8ACAB}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11330,7 +11330,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0D036BDC-A79A-4A0C-96A1-3BC607F585D6}">
+          <x14:cfRule type="dataBar" id="{75A179DD-CD7C-467D-BFEC-3EB09BAEC858}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11343,7 +11343,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D42676F0-B450-4A68-A5EA-A761A52DBE84}">
+          <x14:cfRule type="dataBar" id="{9797D8CE-C476-481A-88E1-78D483D0FE4B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>